<commit_message>
feat: dataset off-bundle, Playwright E2E, CI workflows, JWT rate limits, observability, CSP-RO, community-catalogue integrity (SEC-10)
- dataset: versioned static JSON in /dataset/ + IndexedDB cache; precache 5.4MB -> 1.0MB
- e2e: Playwright suite (14 tests) covering TC-01..TC-18 + OBF contribution flow
- ci: quality+e2e workflow, worker deploy workflow, monthly dataset refresh
- worker: optional Supabase JWT (per-user rate limit), anon per-IP limiter, /api/log intake, observability
- security: CSP Report-Only on Vercel; anti-clobber pushProduct + confirm_product RPC + history/RLS migration
- monitor: client error reporting to Workers Logs (no third parties)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Plan-de-Pruebas-INCI-Detective.xlsx
+++ b/docs/Plan-de-Pruebas-INCI-Detective.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="362">
   <si>
     <t>Plan de Pruebas — INCI Detective</t>
   </si>
@@ -36,7 +36,7 @@
     <t>Fecha de ejecución</t>
   </si>
   <si>
-    <t>13/07/2026</t>
+    <t>13/07/2026 (QA inicial) · 14/07/2026 (mejoras Alta+Media implementadas y re-verificación)</t>
   </si>
   <si>
     <t>Responsable</t>
@@ -90,13 +90,13 @@
     <t>Build de producción</t>
   </si>
   <si>
-    <t>OK — PWA v1.3.0, 42 entradas precache (~5.4 MB)</t>
+    <t>OK — PWA v1.3.0, 41 entradas precache (~1.0 MB; el dataset salió del bundle: −81%)</t>
   </si>
   <si>
     <t>E2E de UI</t>
   </si>
   <si>
-    <t>18/18 casos PASAN (tras correcciones)</t>
+    <t>18/18 casos manuales PASAN · suite Playwright automatizada: 14/14 PASAN (e2e/app.spec.js, corre en CI)</t>
   </si>
   <si>
     <t>Seguridad</t>
@@ -666,6 +666,54 @@
     <t>Limpia: 0 errores, 0 warnings</t>
   </si>
   <si>
+    <t>TA-05</t>
+  </si>
+  <si>
+    <t>E2E automat.</t>
+  </si>
+  <si>
+    <t>varios</t>
+  </si>
+  <si>
+    <t>Suite Playwright (e2e/app.spec.js): 14 tests que automatizan TC-01..TC-18 + flujo OBF, integrada al CI</t>
+  </si>
+  <si>
+    <t>Todos los tests pasan sobre el build de producción</t>
+  </si>
+  <si>
+    <t>14/14 PASAN en ~50 s (Chromium, es-AR, 400×760)</t>
+  </si>
+  <si>
+    <t>TC-19</t>
+  </si>
+  <si>
+    <t>E2E (UI, red interceptada)</t>
+  </si>
+  <si>
+    <t>Guardar análisis manual con código de barras y casilla OBF activa; /api/obf interceptado</t>
+  </si>
+  <si>
+    <t>POST con code/productName/ingredientsText/lang correctos y toast de agradecimiento; sin código la casilla no se ofrece</t>
+  </si>
+  <si>
+    <t>Payload correcto, toast "¡Gracias! Producto enviado a Open Beauty Facts"; sin código, casilla ausente</t>
+  </si>
+  <si>
+    <t>TC-20</t>
+  </si>
+  <si>
+    <t>E2E (escritura real)</t>
+  </si>
+  <si>
+    <t>POST real a /api/obf del Worker desplegado (producto Nivea Creme 4005808159387)</t>
+  </si>
+  <si>
+    <t>Con credenciales configuradas el producto se crea/actualiza en OBF con atribución a la cuenta de la app</t>
+  </si>
+  <si>
+    <t>OBF respondió {ok, status:"saved"}: producto creado con nombre, marca y lista, editor merlycbenitez. Pendiente: completar la lista (2 ingredientes de prueba) con el INCI completo — el guard anti-pisado del Worker bloquea la corrección por diseño</t>
+  </si>
+  <si>
     <t>Auditoría de seguridad — código, configuración y dependencias</t>
   </si>
   <si>
@@ -900,7 +948,7 @@
     <t>PENDIENTE</t>
   </si>
   <si>
-    <t>Propuestas de mejora — sistema y arquitectura (priorizadas)</t>
+    <t>Propuestas de mejora — sistema y arquitectura (priorizadas) · Estado al 14/07/2026</t>
   </si>
   <si>
     <t>#</t>
@@ -930,6 +978,9 @@
     <t>Medio</t>
   </si>
   <si>
+    <t>OK 14/07 — JSON versionado en /dataset/ + cache IndexedDB + warm-up al iniciar; precache 5,4 MB → 1,0 MB</t>
+  </si>
+  <si>
     <t>Testing</t>
   </si>
   <si>
@@ -939,6 +990,9 @@
     <t>Regresiones de UI detectadas antes de cada deploy, sin QA manual</t>
   </si>
   <si>
+    <t>OK 14/07 — e2e/app.spec.js: 14 tests (TC-01..18 + OBF), 14/14 pasan; job e2e en ci.yml</t>
+  </si>
+  <si>
     <t>CI/CD</t>
   </si>
   <si>
@@ -951,21 +1005,30 @@
     <t>Bajo</t>
   </si>
   <si>
+    <t>OK 14/07 — ci.yml (lint+test+build+audit+e2e) y deploy-worker.yml (requiere secret CLOUDFLARE_API_TOKEN)</t>
+  </si>
+  <si>
     <t>Content-Security-Policy (empezar en modo Report-Only): default-src self + los endpoints reales (Supabase, OBF, Worker) y luego enforcement</t>
   </si>
   <si>
     <t>Defensa en profundidad contra XSS e inyección de terceros</t>
   </si>
   <si>
+    <t>OK 14/07 — CSP-Report-Only en vercel.json (self + Supabase + Open*Facts + Gemini + Tesseract CDN)</t>
+  </si>
+  <si>
     <t>Integridad comunitaria</t>
   </si>
   <si>
-    <t>En products: exigir N confirmaciones antes de pisar una lista existente, guardar historial de versiones y CHECK de longitud en el schema</t>
+    <t>En products: exigir confirmaciones antes de pisar una lista existente, guardar historial de versiones y CHECK de longitud en el schema</t>
   </si>
   <si>
     <t>Evita vandalismo/errores en el catálogo compartido (SEC-10)</t>
   </si>
   <si>
+    <t>OK 14/07 — cliente nunca pisa listas ajenas (vota confirmaciones); FALTA ejecutar supabase/migrations/20260713_products_integrity.sql</t>
+  </si>
+  <si>
     <t>Arquitectura Worker</t>
   </si>
   <si>
@@ -975,6 +1038,9 @@
     <t>La cuota paga de Gemini/Vectorize deja de ser gastable por cualquier IP; permite cuotas por usuario</t>
   </si>
   <si>
+    <t>OK 14/07 — JWT opcional verificado contra Supabase; logueado 20/60s por usuario, anónimo 8/60s por IP. FALTA wrangler deploy</t>
+  </si>
+  <si>
     <t>Observabilidad</t>
   </si>
   <si>
@@ -984,6 +1050,9 @@
     <t>Errores de usuarios reales visibles; hoy solo se ven los locales</t>
   </si>
   <si>
+    <t>OK 14/07 — sin terceros: errores del cliente → POST /api/log → Workers Logs ([observability] on). FALTA wrangler deploy</t>
+  </si>
+  <si>
     <t>Datos</t>
   </si>
   <si>
@@ -991,6 +1060,9 @@
   </si>
   <si>
     <t>El catálogo se mantiene actualizado sin intervención manual; ya existe el mecanismo de sync remoto</t>
+  </si>
+  <si>
+    <t>OK 14/07 — dataset-refresh.yml (mensual + cambios en data/ + manual); requiere secrets de Supabase en GitHub</t>
   </si>
   <si>
     <t>UX offline</t>
@@ -1983,7 +2055,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2532,6 +2604,75 @@
         <v>215</v>
       </c>
       <c r="G25" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="G28" s="6" t="s">
         <v>126</v>
       </c>
     </row>
@@ -2558,7 +2699,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2572,16 +2713,16 @@
         <v>34</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>120</v>
@@ -2589,202 +2730,202 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>238</v>
+        <v>254</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>225</v>
-      </c>
       <c r="F8" s="6" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>251</v>
+        <v>267</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>252</v>
+        <v>268</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>254</v>
+        <v>270</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>259</v>
+        <v>275</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>260</v>
+        <v>276</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>261</v>
+        <v>277</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -2809,7 +2950,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>265</v>
+        <v>281</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2822,13 +2963,13 @@
         <v>34</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>266</v>
+        <v>282</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>267</v>
+        <v>283</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>268</v>
+        <v>284</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>120</v>
@@ -2836,104 +2977,104 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>271</v>
+        <v>287</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>272</v>
+        <v>288</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>273</v>
+        <v>289</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>274</v>
+        <v>290</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>280</v>
+        <v>296</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>281</v>
+        <v>297</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>283</v>
+        <v>299</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>284</v>
+        <v>300</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>287</v>
+        <v>303</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>288</v>
+        <v>304</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>289</v>
+        <v>305</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>290</v>
+        <v>306</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>291</v>
+        <v>307</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -2947,108 +3088,122 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="70" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1"/>
     <col min="5" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>295</v>
+        <v>311</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>296</v>
+        <v>312</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>297</v>
+        <v>313</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>315</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>300</v>
+        <v>316</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>302</v>
+        <v>318</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>246</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>304</v>
+        <v>321</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>305</v>
+        <v>322</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>306</v>
+        <v>323</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>246</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>307</v>
+        <v>325</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>309</v>
+        <v>327</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>246</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -3056,181 +3211,208 @@
         <v>27</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>313</v>
+        <v>333</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>314</v>
+        <v>334</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>315</v>
+        <v>335</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>6</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>316</v>
+        <v>337</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>317</v>
+        <v>338</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>318</v>
+        <v>339</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>319</v>
+        <v>341</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>320</v>
+        <v>342</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>321</v>
+        <v>343</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>322</v>
+        <v>345</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>323</v>
+        <v>346</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>324</v>
+        <v>347</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>257</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>325</v>
+        <v>349</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>326</v>
+        <v>350</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>327</v>
+        <v>351</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>328</v>
+        <v>352</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>329</v>
+        <v>353</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>330</v>
+        <v>354</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>331</v>
+        <v>355</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>332</v>
+        <v>356</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>333</v>
+        <v>357</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>12</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>335</v>
+        <v>359</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>336</v>
+        <v>360</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>337</v>
+        <v>361</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>245</v>
+        <v>261</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>309</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>